<commit_message>
test: migrate intake fixtures to declared target-weight template
Drop the Days Since Last Rebalance column from all four portfolio fixtures
in favour of the regenerated upload template's Target Weight % and Purchase
Date columns, so they parse as source: declared with targets summing to 100.
Document the fixture semantics and the template parity in test-data/README.md
and the Portfolio Template section of the README.
</commit_message>
<xml_diff>
--- a/apps/react-client/public/templates/portfolio-template.xlsx
+++ b/apps/react-client/public/templates/portfolio-template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:H4"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -405,6 +405,8 @@
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="20.83203125" customWidth="1"/>
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -426,6 +428,12 @@
       <c r="F1" t="str">
         <v>Current Price</v>
       </c>
+      <c r="G1" t="str">
+        <v>Target Weight %</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Purchase Date</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -446,6 +454,12 @@
       <c r="F2">
         <v>1069.8</v>
       </c>
+      <c r="G2">
+        <v>40</v>
+      </c>
+      <c r="H2" t="str">
+        <v>15-01-2024</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -466,6 +480,12 @@
       <c r="F3">
         <v>195.41</v>
       </c>
+      <c r="G3">
+        <v>25</v>
+      </c>
+      <c r="H3" t="str">
+        <v>02-08-2025</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -486,10 +506,16 @@
       <c r="F4">
         <v>1523.6</v>
       </c>
+      <c r="G4">
+        <v>35</v>
+      </c>
+      <c r="H4" t="str">
+        <v>20-11-2025</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>